<commit_message>
data: hourly update 2026-07-01 14:30Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-01.xlsx
+++ b/data/output/workbook/2026-07-01.xlsx
@@ -611,7 +611,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10353675"/>
+    <ext cx="10125075" cy="10582275"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01 07:25</t>
+          <t>2026-07-01 10:29</t>
         </is>
       </c>
     </row>
@@ -6658,7 +6658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q80"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6675,249 +6675,174 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="29" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="29" t="inlineStr">
         <is>
           <t>Tampa Bay Rays offense vs Kansas City Royals defense</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="30" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B67" s="30" t="inlineStr">
+      <c r="B68" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C67" s="30" t="inlineStr">
+      <c r="C68" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D67" s="30" t="inlineStr">
+      <c r="D68" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E67" s="30" t="inlineStr">
+      <c r="E68" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F67" s="30" t="inlineStr">
+      <c r="F68" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G67" s="30" t="inlineStr">
+      <c r="G68" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H67" s="30" t="inlineStr">
+      <c r="H68" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I67" s="30" t="inlineStr">
+      <c r="I68" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J67" s="30" t="inlineStr">
+      <c r="J68" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K67" s="30" t="inlineStr">
+      <c r="K68" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L67" s="30" t="inlineStr">
+      <c r="L68" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M67" s="30" t="inlineStr">
+      <c r="M68" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N67" s="30" t="inlineStr">
+      <c r="N68" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O67" s="30" t="inlineStr">
+      <c r="O68" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P67" s="30" t="inlineStr">
+      <c r="P68" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q67" s="30" t="inlineStr">
+      <c r="Q68" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B68" s="32" t="n">
-        <v>4.718</v>
-      </c>
-      <c r="C68" s="32" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D68" s="32" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="E68" s="32" t="n">
-        <v>5.067</v>
-      </c>
-      <c r="F68" s="32" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="G68" s="32" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="H68" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I68" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J68" s="34" t="inlineStr">
-        <is>
-          <t>30th</t>
-        </is>
-      </c>
-      <c r="K68" s="32" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="L68" s="32" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="M68" s="32" t="n">
-        <v>6.667</v>
-      </c>
-      <c r="N68" s="32" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="O68" s="32" t="n">
-        <v>5.967</v>
-      </c>
-      <c r="P68" s="32" t="n">
-        <v>5.276</v>
-      </c>
-      <c r="Q68" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B69" s="32" t="n">
-        <v>8.778</v>
+        <v>4.718</v>
       </c>
       <c r="C69" s="32" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="D69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H69" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr"/>
-      <c r="J69" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>4.4</v>
+      </c>
+      <c r="D69" s="32" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="E69" s="32" t="n">
+        <v>5.067</v>
+      </c>
+      <c r="F69" s="32" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G69" s="32" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H69" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I69" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J69" s="34" t="inlineStr">
+        <is>
+          <t>30th</t>
+        </is>
+      </c>
+      <c r="K69" s="32" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="L69" s="32" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="M69" s="32" t="n">
+        <v>6.667</v>
+      </c>
+      <c r="N69" s="32" t="n">
+        <v>6.55</v>
       </c>
       <c r="O69" s="32" t="n">
-        <v>8.800000000000001</v>
+        <v>5.967</v>
       </c>
       <c r="P69" s="32" t="n">
-        <v>8.603999999999999</v>
+        <v>5.276</v>
       </c>
       <c r="Q69" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B70" s="32" t="n">
-        <v>0.956</v>
+        <v>8.778</v>
       </c>
       <c r="C70" s="32" t="n">
-        <v>1.167</v>
+        <v>7.5</v>
       </c>
       <c r="D70" s="32" t="inlineStr">
         <is>
@@ -6970,33 +6895,29 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O70" s="32" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="P70" s="32" t="n">
+        <v>8.603999999999999</v>
       </c>
       <c r="Q70" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>7.244</v>
+        <v>0.956</v>
       </c>
       <c r="C71" s="32" t="n">
-        <v>7.667</v>
+        <v>1.167</v>
       </c>
       <c r="D71" s="32" t="inlineStr">
         <is>
@@ -7049,320 +6970,324 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O71" s="32" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="P71" s="32" t="n">
-        <v>8.208</v>
+      <c r="O71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B72" s="32" t="n">
+        <v>7.244</v>
+      </c>
+      <c r="C72" s="32" t="n">
+        <v>7.667</v>
+      </c>
+      <c r="D72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="inlineStr"/>
+      <c r="J72" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O72" s="32" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P72" s="32" t="n">
+        <v>8.208</v>
+      </c>
+      <c r="Q72" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B72" s="32" t="n">
+      <c r="B73" s="32" t="n">
         <v>0.536</v>
       </c>
-      <c r="C72" s="32" t="n">
+      <c r="C73" s="32" t="n">
         <v>0.633</v>
       </c>
-      <c r="D72" s="32" t="n">
+      <c r="D73" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="E72" s="32" t="n">
+      <c r="E73" s="32" t="n">
         <v>0.733</v>
       </c>
-      <c r="F72" s="32" t="n">
+      <c r="F73" s="32" t="n">
         <v>0.9</v>
       </c>
-      <c r="G72" s="32" t="n">
+      <c r="G73" s="32" t="n">
         <v>1.4</v>
       </c>
-      <c r="H72" s="33" t="inlineStr">
+      <c r="H73" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I72" s="32" t="inlineStr">
+      <c r="I73" s="32" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="J72" s="34" t="inlineStr">
+      <c r="J73" s="34" t="inlineStr">
         <is>
           <t>24th</t>
         </is>
       </c>
-      <c r="K72" s="32" t="n">
+      <c r="K73" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="L72" s="32" t="n">
+      <c r="L73" s="32" t="n">
         <v>1.1</v>
       </c>
-      <c r="M72" s="32" t="n">
+      <c r="M73" s="32" t="n">
         <v>0.867</v>
       </c>
-      <c r="N72" s="32" t="n">
+      <c r="N73" s="32" t="n">
         <v>1.15</v>
       </c>
-      <c r="O72" s="32" t="n">
+      <c r="O73" s="32" t="n">
         <v>1.133</v>
       </c>
-      <c r="P72" s="32" t="n">
+      <c r="P73" s="32" t="n">
         <v>0.822</v>
       </c>
-      <c r="Q72" s="35" t="inlineStr">
+      <c r="Q73" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="29" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="29" t="inlineStr">
         <is>
           <t>Kansas City Royals offense vs Tampa Bay Rays defense</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="30" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B75" s="30" t="inlineStr">
+      <c r="B76" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C75" s="30" t="inlineStr">
+      <c r="C76" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D75" s="30" t="inlineStr">
+      <c r="D76" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E75" s="30" t="inlineStr">
+      <c r="E76" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F75" s="30" t="inlineStr">
+      <c r="F76" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G75" s="30" t="inlineStr">
+      <c r="G76" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H75" s="30" t="inlineStr">
+      <c r="H76" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I75" s="30" t="inlineStr">
+      <c r="I76" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J75" s="30" t="inlineStr">
+      <c r="J76" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K75" s="30" t="inlineStr">
+      <c r="K76" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L75" s="30" t="inlineStr">
+      <c r="L76" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M75" s="30" t="inlineStr">
+      <c r="M76" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N75" s="30" t="inlineStr">
+      <c r="N76" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O75" s="30" t="inlineStr">
+      <c r="O76" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P75" s="30" t="inlineStr">
+      <c r="P76" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q75" s="30" t="inlineStr">
+      <c r="Q76" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B76" s="32" t="n">
-        <v>4.211</v>
-      </c>
-      <c r="C76" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="D76" s="32" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="E76" s="32" t="n">
-        <v>5.133</v>
-      </c>
-      <c r="F76" s="32" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G76" s="32" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="H76" s="34" t="inlineStr">
-        <is>
-          <t>26th</t>
-        </is>
-      </c>
-      <c r="I76" s="32" t="inlineStr"/>
-      <c r="J76" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K76" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="L76" s="32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="M76" s="32" t="n">
-        <v>3.267</v>
-      </c>
-      <c r="N76" s="32" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="O76" s="32" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="P76" s="32" t="n">
-        <v>4.493</v>
-      </c>
-      <c r="Q76" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B77" s="32" t="n">
-        <v>7.792</v>
+        <v>4.211</v>
       </c>
       <c r="C77" s="32" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="D77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>5</v>
+      </c>
+      <c r="D77" s="32" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="E77" s="32" t="n">
+        <v>5.133</v>
+      </c>
+      <c r="F77" s="32" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G77" s="32" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H77" s="34" t="inlineStr">
+        <is>
+          <t>26th</t>
         </is>
       </c>
       <c r="I77" s="32" t="inlineStr"/>
-      <c r="J77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J77" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K77" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L77" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M77" s="32" t="n">
+        <v>3.267</v>
+      </c>
+      <c r="N77" s="32" t="n">
+        <v>3.5</v>
       </c>
       <c r="O77" s="32" t="n">
-        <v>11.667</v>
+        <v>4.5</v>
       </c>
       <c r="P77" s="32" t="n">
-        <v>8.467000000000001</v>
+        <v>4.493</v>
       </c>
       <c r="Q77" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B78" s="32" t="n">
-        <v>0.896</v>
+        <v>7.792</v>
       </c>
       <c r="C78" s="32" t="n">
-        <v>1</v>
+        <v>8.6</v>
       </c>
       <c r="D78" s="32" t="inlineStr">
         <is>
@@ -7415,33 +7340,29 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O78" s="32" t="n">
+        <v>11.667</v>
+      </c>
+      <c r="P78" s="32" t="n">
+        <v>8.467000000000001</v>
       </c>
       <c r="Q78" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>8.021000000000001</v>
+        <v>0.896</v>
       </c>
       <c r="C79" s="32" t="n">
-        <v>8.4</v>
+        <v>1</v>
       </c>
       <c r="D79" s="32" t="inlineStr">
         <is>
@@ -7494,76 +7415,155 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O79" s="32" t="n">
-        <v>6.667</v>
-      </c>
-      <c r="P79" s="32" t="n">
-        <v>7.778</v>
+      <c r="O79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>8.021000000000001</v>
+      </c>
+      <c r="C80" s="32" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr"/>
+      <c r="J80" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O80" s="32" t="n">
+        <v>6.667</v>
+      </c>
+      <c r="P80" s="32" t="n">
+        <v>7.778</v>
+      </c>
+      <c r="Q80" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B80" s="32" t="n">
+      <c r="B81" s="32" t="n">
         <v>0.466</v>
       </c>
-      <c r="C80" s="32" t="n">
+      <c r="C81" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="D80" s="32" t="n">
+      <c r="D81" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="E80" s="32" t="n">
+      <c r="E81" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="F80" s="32" t="n">
+      <c r="F81" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="G80" s="32" t="n">
+      <c r="G81" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="H80" s="36" t="inlineStr">
+      <c r="H81" s="36" t="inlineStr">
         <is>
           <t>14th</t>
         </is>
       </c>
-      <c r="I80" s="32" t="inlineStr">
+      <c r="I81" s="32" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="J80" s="36" t="inlineStr">
+      <c r="J81" s="36" t="inlineStr">
         <is>
           <t>20th</t>
         </is>
       </c>
-      <c r="K80" s="32" t="n">
+      <c r="K81" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="L80" s="32" t="n">
+      <c r="L81" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="M80" s="32" t="n">
+      <c r="M81" s="32" t="n">
         <v>0.333</v>
       </c>
-      <c r="N80" s="32" t="n">
+      <c r="N81" s="32" t="n">
         <v>0.35</v>
       </c>
-      <c r="O80" s="32" t="n">
+      <c r="O81" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="P80" s="32" t="n">
+      <c r="P81" s="32" t="n">
         <v>0.493</v>
       </c>
-      <c r="Q80" s="35" t="inlineStr">
+      <c r="Q81" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8584,7 +8584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8724,17 +8724,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6595269230769231</v>
+        <v>0.6154411764705883</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-194</v>
+        <v>-160</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-108</v>
+        <v>104</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 66.0% (fair -194). Your call.</t>
+          <t>Model 61.5% (fair -160). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8836,37 +8836,37 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
+          <t>Atlanta Dream @ Washington Mystics</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Under 12</t>
+          <t>Washington Mystics</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5816097560975609</v>
+        <v>0.3552321981424149</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-139</v>
+        <v>182</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>105</v>
+        <v>223</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 35.5% (fair +182). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8907,12 +8907,12 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Washington Mystics</t>
+          <t>Los Angeles Angels @ Seattle Mariners</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -8922,17 +8922,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3510810810810811</v>
+        <v>0.3901748251748251</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>233</v>
+        <v>186</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 35.1% (fair +185). Your call.</t>
+          <t>Model 39.0% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8973,32 +8973,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Seattle Mariners</t>
+          <t>Atlanta Dream @ Washington Mystics</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Washington Mystics +6.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3996402877697841</v>
+        <v>0.5619058823529411</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>150</v>
+        <v>-128</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>178</v>
+        <v>-104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9022,7 +9022,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 40.0% (fair +150). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9039,32 +9039,32 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Minnesota Twins @ Houston Astros</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Under 10</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5475</v>
+        <v>0.4870403587443947</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-121</v>
+        <v>105</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9088,7 +9088,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9105,32 +9105,32 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Washington Mystics</t>
+          <t>San Diego Padres @ Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>02:10</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics +6.5</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5551764705882353</v>
+        <v>0.4226953125</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-125</v>
+        <v>137</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-104</v>
+        <v>156</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9154,7 +9154,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 42.3% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9171,12 +9171,12 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Los Angeles Dodgers</t>
+          <t>Chicago White Sox @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -9186,17 +9186,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.425234375</v>
+        <v>0.5499254901960784</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>135</v>
+        <v>-122</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>156</v>
+        <v>-104</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9237,12 +9237,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Phoenix Mercury</t>
+          <t>Dallas Wings @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -9252,17 +9252,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm +6.5</t>
+          <t>Connecticut Sun +8.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5319607843137254</v>
+        <v>0.5634619047619048</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-114</v>
+        <v>-129</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>104</v>
+        <v>-110</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9298,37 +9298,37 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Houston Astros</t>
+          <t>Seattle Storm @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4877477477477478</v>
+        <v>0.5</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -9352,7 +9352,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 50.0% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9369,12 +9369,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Cleveland Guardians</t>
+          <t>Seattle Storm @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -9384,17 +9384,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Seattle Storm</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5554730769230769</v>
+        <v>0.3539666666666667</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-125</v>
+        <v>183</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-108</v>
+        <v>200</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9418,7 +9418,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 35.4% (fair +183). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9430,37 +9430,37 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings @ Connecticut Sun</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun +8.5</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5581714285714287</v>
+        <v>0.4655506607929515</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-126</v>
+        <v>115</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-110</v>
+        <v>127</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9484,7 +9484,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9496,37 +9496,37 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Houston Astros</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5306</v>
+        <v>0.4736486486486488</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-113</v>
+        <v>111</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -9550,7 +9550,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -9567,12 +9567,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Phoenix Mercury</t>
+          <t>Cincinnati Reds @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -9582,17 +9582,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.353</v>
+        <v>0.6614259259259259</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>183</v>
+        <v>-195</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>200</v>
+        <v>-170</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 35.3% (fair +183). Your call.</t>
+          <t>Model 66.1% (fair -195). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9628,17 +9628,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>St. Louis Cardinals @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9648,17 +9648,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>St. Louis Cardinals</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6604185185185184</v>
+        <v>0.4700900900900902</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-194</v>
+        <v>113</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-170</v>
+        <v>122</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 66.0% (fair -194). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9694,17 +9694,17 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9714,17 +9714,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4724324324324325</v>
+        <v>0.4596916299559472</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9748,7 +9748,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 47.2% (fair +112). Your call.</t>
+          <t>Model 46.0% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9760,7 +9760,7 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -9784,13 +9784,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4650222222222222</v>
+        <v>0.4862910798122066</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9826,37 +9826,37 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Phoenix Mercury</t>
+          <t>San Diego Padres @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5468047619047619</v>
+        <v>0.4779629629629629</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-121</v>
+        <v>109</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-110</v>
+        <v>116</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9880,7 +9880,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -9897,12 +9897,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -9912,17 +9912,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4591189427312775</v>
+        <v>0.4646846846846848</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 46.5% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -9963,12 +9963,12 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -9978,17 +9978,17 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4588105726872247</v>
+        <v>0.5126500000000001</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>118</v>
+        <v>-105</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10012,7 +10012,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10021,273 +10021,9 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>18:20</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>San Diego Padres</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="n">
-        <v>0.4762672811059908</v>
-      </c>
-      <c r="G25" s="14" t="n">
-        <v>110</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v>117</v>
-      </c>
-      <c r="I25" s="13">
-        <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
-        <v/>
-      </c>
-      <c r="J25" s="16">
-        <f>IF($H$25="","",$F$25*IF($H$25&lt;0,-100/$H$25,$H$25/100)-(1-$F$25))</f>
-        <v/>
-      </c>
-      <c r="K25" s="17">
-        <f>IF($H$25="","",MAX(0,($F$25*IF($H$25&lt;0,-100/$H$25,$H$25/100)-(1-$F$25))/IF($H$25&lt;0,-100/$H$25,$H$25/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L25" s="18">
-        <f>IF($H$25="","",ROUND(MIN($K$25,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M25" s="12">
-        <f>IF($J$25="","",IF($J$25&lt;0,"Pass",IF($J$25&lt;'Settings'!$B$4,"Thin",IF($J$25&lt;0.06,"✅ Sharp band",IF($J$25&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N25" s="19" t="inlineStr">
-        <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
-        </is>
-      </c>
-      <c r="O25" s="15" t="n"/>
-      <c r="P25" s="16">
-        <f>IF(OR($H$25="",$O$25=""),"",(1+IF($H$25&lt;0,-100/$H$25,$H$25/100))/(1+IF($O$25&lt;0,-100/$O$25,$O$25/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="C26" s="20" t="inlineStr">
-        <is>
-          <t>23:40</t>
-        </is>
-      </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>0.4646846846846848</v>
-      </c>
-      <c r="G26" s="14" t="n">
-        <v>115</v>
-      </c>
-      <c r="H26" s="15" t="n">
-        <v>122</v>
-      </c>
-      <c r="I26" s="13">
-        <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
-        <v/>
-      </c>
-      <c r="J26" s="16">
-        <f>IF($H$26="","",$F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))</f>
-        <v/>
-      </c>
-      <c r="K26" s="17">
-        <f>IF($H$26="","",MAX(0,($F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))/IF($H$26&lt;0,-100/$H$26,$H$26/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L26" s="18">
-        <f>IF($H$26="","",ROUND(MIN($K$26,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M26" s="12">
-        <f>IF($J$26="","",IF($J$26&lt;0,"Pass",IF($J$26&lt;'Settings'!$B$4,"Thin",IF($J$26&lt;0.06,"✅ Sharp band",IF($J$26&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N26" s="19" t="inlineStr">
-        <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
-        </is>
-      </c>
-      <c r="O26" s="15" t="n"/>
-      <c r="P26" s="16">
-        <f>IF(OR($H$26="",$O$26=""),"",(1+IF($H$26&lt;0,-100/$H$26,$H$26/100))/(1+IF($O$26&lt;0,-100/$O$26,$O$26/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>17:10</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="F27" s="13" t="n">
-        <v>0.51165</v>
-      </c>
-      <c r="G27" s="14" t="n">
-        <v>-105</v>
-      </c>
-      <c r="H27" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="I27" s="13">
-        <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
-        <v/>
-      </c>
-      <c r="J27" s="16">
-        <f>IF($H$27="","",$F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))</f>
-        <v/>
-      </c>
-      <c r="K27" s="17">
-        <f>IF($H$27="","",MAX(0,($F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))/IF($H$27&lt;0,-100/$H$27,$H$27/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L27" s="18">
-        <f>IF($H$27="","",ROUND(MIN($K$27,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M27" s="12">
-        <f>IF($J$27="","",IF($J$27&lt;0,"Pass",IF($J$27&lt;'Settings'!$B$4,"Thin",IF($J$27&lt;0.06,"✅ Sharp band",IF($J$27&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N27" s="19" t="inlineStr">
-        <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
-        </is>
-      </c>
-      <c r="O27" s="15" t="n"/>
-      <c r="P27" s="16">
-        <f>IF(OR($H$27="",$O$27=""),"",(1+IF($H$27&lt;0,-100/$H$27,$H$27/100))/(1+IF($O$27&lt;0,-100/$O$27,$O$27/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="inlineStr">
-        <is>
-          <t>Detroit Tigers @ Texas Rangers</t>
-        </is>
-      </c>
-      <c r="C28" s="20" t="inlineStr">
-        <is>
-          <t>00:05</t>
-        </is>
-      </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E28" s="20" t="inlineStr">
-        <is>
-          <t>Detroit Tigers</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.4796713615023475</v>
-      </c>
-      <c r="G28" s="14" t="n">
-        <v>108</v>
-      </c>
-      <c r="H28" s="15" t="n">
-        <v>113</v>
-      </c>
-      <c r="I28" s="13">
-        <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
-        <v/>
-      </c>
-      <c r="J28" s="16">
-        <f>IF($H$28="","",$F$28*IF($H$28&lt;0,-100/$H$28,$H$28/100)-(1-$F$28))</f>
-        <v/>
-      </c>
-      <c r="K28" s="17">
-        <f>IF($H$28="","",MAX(0,($F$28*IF($H$28&lt;0,-100/$H$28,$H$28/100)-(1-$F$28))/IF($H$28&lt;0,-100/$H$28,$H$28/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L28" s="18">
-        <f>IF($H$28="","",ROUND(MIN($K$28,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M28" s="12">
-        <f>IF($J$28="","",IF($J$28&lt;0,"Pass",IF($J$28&lt;'Settings'!$B$4,"Thin",IF($J$28&lt;0.06,"✅ Sharp band",IF($J$28&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N28" s="19" t="inlineStr">
-        <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
-        </is>
-      </c>
-      <c r="O28" s="15" t="n"/>
-      <c r="P28" s="16">
-        <f>IF(OR($H$28="",$O$28=""),"",(1+IF($H$28&lt;0,-100/$H$28,$H$28/100))/(1+IF($O$28&lt;0,-100/$O$28,$O$28/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J28">
+  <conditionalFormatting sqref="J5:J24">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -10453,10 +10189,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4591189427312775</v>
+        <v>0.4655506607929515</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>127</v>
@@ -10483,7 +10219,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -10519,10 +10255,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5408409691629956</v>
+        <v>0.5344629955947137</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-118</v>
+        <v>-115</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-127</v>
@@ -10549,7 +10285,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10585,13 +10321,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4595</v>
+        <v>0.4757</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -10615,7 +10351,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +118). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10651,13 +10387,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5405</v>
+        <v>0.5243</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -10681,7 +10417,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -118). Your call.</t>
+          <t>Model 52.4% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10717,10 +10453,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3826</v>
+        <v>0.3639</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>150</v>
@@ -10747,7 +10483,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 36.4% (fair +175). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10783,10 +10519,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6173999999999999</v>
+        <v>0.6361</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-161</v>
+        <v>-175</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>144</v>
@@ -10813,7 +10549,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 63.6% (fair -175). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -10849,7 +10585,7 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.51165</v>
+        <v>0.5126500000000001</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>-105</v>
@@ -10879,7 +10615,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10915,13 +10651,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4883411764705882</v>
+        <v>0.4873472906403941</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>105</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-104</v>
+        <v>-103</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -10945,7 +10681,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10981,13 +10717,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4976</v>
+        <v>0.4877</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -11011,7 +10747,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 48.8% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -11047,13 +10783,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5024</v>
+        <v>0.5123</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-101</v>
+        <v>-105</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -11077,7 +10813,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -11113,10 +10849,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.326</v>
+        <v>0.3244</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>180</v>
@@ -11143,7 +10879,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 32.6% (fair +207). Your call.</t>
+          <t>Model 32.4% (fair +208). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -11179,13 +10915,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6739999999999999</v>
+        <v>0.6756</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-207</v>
+        <v>-208</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -11209,7 +10945,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 67.4% (fair -207). Your call.</t>
+          <t>Model 67.6% (fair -208). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -11251,7 +10987,7 @@
         <v>100</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -11383,7 +11119,7 @@
         <v>157</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -11449,7 +11185,7 @@
         <v>-157</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -11641,13 +11377,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.444625550660793</v>
+        <v>0.4454222222222222</v>
       </c>
       <c r="G23" s="14" t="n">
         <v>125</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -11707,10 +11443,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5553872246696036</v>
+        <v>0.5545480176211454</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-125</v>
+        <v>-124</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>-127</v>
@@ -11737,7 +11473,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 55.5% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11769,17 +11505,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 10</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4525365853658537</v>
+        <v>0.4444</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -11803,7 +11539,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -11835,17 +11571,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 10</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5475</v>
+        <v>0.5556</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-121</v>
+        <v>-125</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -11869,7 +11605,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -11905,10 +11641,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4153</v>
+        <v>0.411</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>150</v>
@@ -11935,7 +11671,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 41.1% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -11971,13 +11707,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5847</v>
+        <v>0.589</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-141</v>
+        <v>-143</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-111</v>
+        <v>-113</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -12001,7 +11737,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -12037,13 +11773,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4762672811059908</v>
+        <v>0.4779629629629629</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -12067,7 +11803,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12103,10 +11839,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5237185185185185</v>
+        <v>0.5220537037037037</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-110</v>
+        <v>-109</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-116</v>
@@ -12133,7 +11869,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -12165,17 +11901,17 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Over 12</t>
+          <t>Over 12.5</t>
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4184121951219512</v>
+        <v>0.2438</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>139</v>
+        <v>310</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-105</v>
+        <v>113</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -12199,7 +11935,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 24.4% (fair +310). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12231,14 +11967,14 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>Under 12</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5816097560975609</v>
+        <v>0.7562</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-139</v>
+        <v>-310</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>105</v>
@@ -12265,7 +12001,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 75.6% (fair -310). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -12301,13 +12037,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.3694</v>
+        <v>0.3672</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -12331,7 +12067,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 36.9% (fair +171). Your call.</t>
+          <t>Model 36.7% (fair +172). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -12367,10 +12103,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.6306</v>
+        <v>0.6328</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-171</v>
+        <v>-172</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>163</v>
@@ -12397,7 +12133,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 63.1% (fair -171). Your call.</t>
+          <t>Model 63.3% (fair -172). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -12433,13 +12169,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.5148173076923077</v>
+        <v>0.5120980392156862</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -12463,7 +12199,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -12499,10 +12235,10 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4851960784313725</v>
+        <v>0.4879411764705882</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H36" s="15" t="n">
         <v>104</v>
@@ -12529,7 +12265,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 48.8% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -12565,13 +12301,13 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.3967</v>
+        <v>0.4037</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>113</v>
+        <v>-104</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -12595,7 +12331,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 39.7% (fair +152). Your call.</t>
+          <t>Model 40.4% (fair +148). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -12631,13 +12367,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.6032999999999999</v>
+        <v>0.5963000000000001</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-152</v>
+        <v>-148</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -12661,7 +12397,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 60.3% (fair -152). Your call.</t>
+          <t>Model 59.6% (fair -148). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -12697,7 +12433,7 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.4588105726872247</v>
+        <v>0.4596916299559472</v>
       </c>
       <c r="G39" s="14" t="n">
         <v>118</v>
@@ -12727,7 +12463,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 46.0% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12763,13 +12499,13 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5411766519823789</v>
+        <v>0.5403353711790393</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>-118</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>-127</v>
+        <v>-129</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -12793,7 +12529,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -12825,17 +12561,17 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.5709</v>
+        <v>0.5766</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>-133</v>
+        <v>-136</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -12859,7 +12595,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 57.1% (fair -133). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -12891,17 +12627,17 @@
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4291</v>
+        <v>0.4234</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -12925,7 +12661,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 42.9% (fair +133). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -12961,13 +12697,13 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.3746</v>
+        <v>0.3733</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -12991,7 +12727,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 37.5% (fair +167). Your call.</t>
+          <t>Model 37.3% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -13027,13 +12763,13 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.6254</v>
+        <v>0.6267</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>-167</v>
+        <v>-168</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>-117</v>
+        <v>-116</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -13057,7 +12793,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 62.5% (fair -167). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -13093,13 +12829,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.4650222222222222</v>
+        <v>0.4700900900900902</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -13123,7 +12859,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -13159,13 +12895,13 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.5349665198237886</v>
+        <v>0.5299306306306306</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-127</v>
+        <v>-122</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -13189,7 +12925,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -13231,7 +12967,7 @@
         <v>158</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -13297,7 +13033,7 @@
         <v>-158</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -13363,7 +13099,7 @@
         <v>179</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -13429,7 +13165,7 @@
         <v>-179</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>-114</v>
+        <v>-119</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -13617,17 +13353,17 @@
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>Over 10.5</t>
+          <t>Over 11</t>
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.3922</v>
+        <v>0.3048</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>155</v>
+        <v>228</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -13651,7 +13387,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 39.2% (fair +155). Your call.</t>
+          <t>Model 30.5% (fair +228). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -13683,17 +13419,17 @@
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Under 11</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.6078</v>
+        <v>0.6952</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-155</v>
+        <v>-228</v>
       </c>
       <c r="H54" s="15" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="I54" s="13">
         <f>IF($H$54="","",IF($H$54&lt;0,-$H$54/(-$H$54+100),100/($H$54+100)))</f>
@@ -13717,7 +13453,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 69.5% (fair -228). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -13753,13 +13489,13 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.4877477477477478</v>
+        <v>0.4870403587443947</v>
       </c>
       <c r="G55" s="14" t="n">
         <v>105</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -13783,7 +13519,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -13819,7 +13555,7 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5122351351351352</v>
+        <v>0.5130045045045045</v>
       </c>
       <c r="G56" s="14" t="n">
         <v>-105</v>
@@ -13849,7 +13585,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -13881,17 +13617,17 @@
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.5306</v>
+        <v>0.474</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>-113</v>
+        <v>111</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -13915,7 +13651,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -13947,14 +13683,14 @@
       </c>
       <c r="E58" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.4694146341463415</v>
+        <v>0.526</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>113</v>
+        <v>-111</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>105</v>
@@ -13981,7 +13717,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 46.9% (fair +113). Your call.</t>
+          <t>Model 52.6% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14023,7 +13759,7 @@
         <v>209</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -14089,7 +13825,7 @@
         <v>-209</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>-125</v>
+        <v>-123</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -14793,10 +14529,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.3395925925925926</v>
+        <v>0.3385555555555556</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H71" s="15" t="n">
         <v>170</v>
@@ -14823,7 +14559,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 34.0% (fair +194). Your call.</t>
+          <t>Model 33.9% (fair +195). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -14859,10 +14595,10 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.6604185185185184</v>
+        <v>0.6614259259259259</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>-194</v>
+        <v>-195</v>
       </c>
       <c r="H72" s="15" t="n">
         <v>-170</v>
@@ -14889,7 +14625,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 66.0% (fair -194). Your call.</t>
+          <t>Model 66.1% (fair -195). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -14925,10 +14661,10 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.555611013215859</v>
+        <v>0.5542123348017621</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-125</v>
+        <v>-124</v>
       </c>
       <c r="H73" s="15" t="n">
         <v>-127</v>
@@ -14955,7 +14691,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 55.4% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -14991,10 +14727,10 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.4444052863436123</v>
+        <v>0.4457709251101322</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H74" s="15" t="n">
         <v>127</v>
@@ -15021,7 +14757,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 44.6% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -15057,13 +14793,13 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.5554730769230769</v>
+        <v>0.5499254901960784</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="H75" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I75" s="13">
         <f>IF($H$75="","",IF($H$75&lt;0,-$H$75/(-$H$75+100),100/($H$75+100)))</f>
@@ -15087,7 +14823,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -15123,10 +14859,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.4445098039215686</v>
+        <v>0.4500980392156863</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>104</v>
@@ -15153,7 +14889,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +125). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -15189,13 +14925,13 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.4901442307692308</v>
+        <v>0.4862910798122066</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H77" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I77" s="13">
         <f>IF($H$77="","",IF($H$77&lt;0,-$H$77/(-$H$77+100),100/($H$77+100)))</f>
@@ -15219,7 +14955,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -15255,10 +14991,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.5098793427230046</v>
+        <v>0.5136990610328639</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>-104</v>
+        <v>-106</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>-113</v>
@@ -15285,7 +15021,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 51.4% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -15321,10 +15057,10 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.5275783410138248</v>
+        <v>0.5263921658986175</v>
       </c>
       <c r="G79" s="14" t="n">
-        <v>-112</v>
+        <v>-111</v>
       </c>
       <c r="H79" s="15" t="n">
         <v>-117</v>
@@ -15351,7 +15087,7 @@
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>Model 52.8% (fair -112). Your call.</t>
+          <t>Model 52.6% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O79" s="15" t="n"/>
@@ -15387,10 +15123,10 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.4724324324324325</v>
+        <v>0.4736486486486488</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H80" s="15" t="n">
         <v>122</v>
@@ -15417,7 +15153,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 47.2% (fair +112). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -15453,13 +15189,13 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.4796713615023475</v>
+        <v>0.5036</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>108</v>
+        <v>-101</v>
       </c>
       <c r="H81" s="15" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="I81" s="13">
         <f>IF($H$81="","",IF($H$81&lt;0,-$H$81/(-$H$81+100),100/($H$81+100)))</f>
@@ -15483,7 +15219,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 50.4% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -15519,13 +15255,13 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.5202995391705069</v>
+        <v>0.4964</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>-108</v>
+        <v>101</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="I82" s="13">
         <f>IF($H$82="","",IF($H$82&lt;0,-$H$82/(-$H$82+100),100/($H$82+100)))</f>
@@ -15549,7 +15285,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 49.6% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -15585,13 +15321,13 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.3996402877697841</v>
+        <v>0.3901748251748251</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="H83" s="15" t="n">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="I83" s="13">
         <f>IF($H$83="","",IF($H$83&lt;0,-$H$83/(-$H$83+100),100/($H$83+100)))</f>
@@ -15615,7 +15351,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 40.0% (fair +150). Your call.</t>
+          <t>Model 39.0% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15651,13 +15387,13 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.6003518518518518</v>
+        <v>0.6098328671328671</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-150</v>
+        <v>-156</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>-170</v>
+        <v>-186</v>
       </c>
       <c r="I84" s="13">
         <f>IF($H$84="","",IF($H$84&lt;0,-$H$84/(-$H$84+100),100/($H$84+100)))</f>
@@ -15681,7 +15417,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 60.0% (fair -150). Your call.</t>
+          <t>Model 61.0% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -15717,10 +15453,10 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.425234375</v>
+        <v>0.4226953125</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H85" s="15" t="n">
         <v>156</v>
@@ -15747,7 +15483,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 42.3% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -15783,10 +15519,10 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.5747625000000001</v>
+        <v>0.5772609375000001</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>-135</v>
+        <v>-137</v>
       </c>
       <c r="H86" s="15" t="n">
         <v>-156</v>
@@ -15813,7 +15549,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 57.5% (fair -135). Your call.</t>
+          <t>Model 57.7% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -15990,13 +15726,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6489176470588235</v>
+        <v>0.6447732732732733</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-185</v>
+        <v>-182</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-240</v>
+        <v>-233</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -16020,7 +15756,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 64.9% (fair -185). Your call.</t>
+          <t>Model 64.5% (fair -182). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -16056,13 +15792,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.3510810810810811</v>
+        <v>0.3552321981424149</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -16086,7 +15822,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 35.1% (fair +185). Your call.</t>
+          <t>Model 35.5% (fair +182). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -16118,17 +15854,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6595269230769231</v>
+        <v>0.6154411764705883</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-194</v>
+        <v>-160</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-108</v>
+        <v>104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -16152,7 +15888,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 66.0% (fair -194). Your call.</t>
+          <t>Model 61.5% (fair -160). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -16184,17 +15920,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 165.5</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3405</v>
+        <v>0.3846000000000001</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>194</v>
+        <v>160</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-108</v>
+        <v>104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -16218,7 +15954,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 34.1% (fair +194). Your call.</t>
+          <t>Model 38.5% (fair +160). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -16254,10 +15990,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5551764705882353</v>
+        <v>0.5619058823529411</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-125</v>
+        <v>-128</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>-104</v>
@@ -16284,7 +16020,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -16320,13 +16056,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4448</v>
+        <v>0.4381042654028435</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -16350,7 +16086,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +125). Your call.</t>
+          <t>Model 43.8% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -16514,17 +16250,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 171.5</t>
+          <t>Over 172.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.442252380952381</v>
+        <v>0.4191079812206573</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-110</v>
+        <v>113</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -16548,7 +16284,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 41.9% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -16580,17 +16316,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 171.5</t>
+          <t>Under 172.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5578000000000001</v>
+        <v>0.5809</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-126</v>
+        <v>-139</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-110</v>
+        <v>113</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -16614,7 +16350,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 58.1% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -16650,10 +16386,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5581714285714287</v>
+        <v>0.5634619047619048</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-126</v>
+        <v>-129</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>-110</v>
@@ -16680,7 +16416,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -16716,13 +16452,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4418269230769231</v>
+        <v>0.4365437788018434</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -16746,7 +16482,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -16782,7 +16518,7 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.353</v>
+        <v>0.3539666666666667</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>183</v>
@@ -16812,7 +16548,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 35.3% (fair +183). Your call.</t>
+          <t>Model 35.4% (fair +183). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -16848,13 +16584,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.6469829431438127</v>
+        <v>0.6460727891156463</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>-183</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-199</v>
+        <v>-194</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -16878,7 +16614,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 64.7% (fair -183). Your call.</t>
+          <t>Model 64.6% (fair -183). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -16910,17 +16646,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5468047619047619</v>
+        <v>0.5</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-121</v>
+        <v>100</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-110</v>
+        <v>113</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -16944,7 +16680,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 50.0% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -16976,17 +16712,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 168.5</t>
+          <t>Under 170.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4532</v>
+        <v>0.5</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-110</v>
+        <v>113</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -17010,7 +16746,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 50.0% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -17046,13 +16782,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4680509803921569</v>
+        <v>0.4263</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -17076,7 +16812,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 42.6% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -17112,10 +16848,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5319607843137254</v>
+        <v>0.5737</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-114</v>
+        <v>-135</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>104</v>
@@ -17142,7 +16878,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 57.4% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>

</xml_diff>